<commit_message>
deployment of mallcom shoes qa done and updated in the deployment matrix
</commit_message>
<xml_diff>
--- a/deployment matrix/Deployment Matrix For Frontend.xlsx
+++ b/deployment matrix/Deployment Matrix For Frontend.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yash.kesharwani\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DevOps\VFlow_Frontend\vflow-frontend\deployment matrix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1ABA7D5A-4978-43A7-AFD7-50E2857C4A6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDE00146-8440-40D4-AC75-2232D35C5449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Matrix For Frontend" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
   <si>
     <t>Date</t>
   </si>
@@ -68,12 +68,18 @@
   </si>
   <si>
     <t>Done</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Task 6771: MTO Update logic of forget password page and site specific client name display feature</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -210,7 +216,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -388,6 +394,18 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -551,9 +569,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -908,9 +928,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="57.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -972,10 +1006,40 @@
       <c r="G2" t="s">
         <v>14</v>
       </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="3"/>
       <c r="J2">
         <v>2</v>
       </c>
       <c r="L2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
+        <v>45645</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="3"/>
+      <c r="L3" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated the deployment matrix
</commit_message>
<xml_diff>
--- a/deployment matrix/Deployment Matrix For Frontend.xlsx
+++ b/deployment matrix/Deployment Matrix For Frontend.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tarun.shetty\Desktop\VFlow\vflow-frontend\deployment matrix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB51EAC9-D566-4D58-9FF6-0EBFD78F5FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B1FC74-C841-4D30-A956-680448F82B99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
   <si>
     <t>Date</t>
   </si>
@@ -80,9 +80,6 @@
   </si>
   <si>
     <t>Tarun</t>
-  </si>
-  <si>
-    <t>Pivot mode in bm report</t>
   </si>
   <si>
     <t>Pending</t>
@@ -1066,7 +1063,7 @@
         <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
         <v>14</v>
@@ -1083,7 +1080,7 @@
         <v>2</v>
       </c>
       <c r="L4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
minor changes in the frontend
</commit_message>
<xml_diff>
--- a/deployment matrix/Deployment Matrix For Frontend.xlsx
+++ b/deployment matrix/Deployment Matrix For Frontend.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tarun.shetty\Desktop\VFlow\vflow-frontend\deployment matrix\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DevOps\VFlow_Frontend\vflow-frontend\deployment matrix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3000B97-4D5B-4669-9D38-4B4E669E247C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1425B4CF-16A7-44A4-8121-7AECDD01F381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Matrix For Frontend" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="24">
   <si>
     <t>Date</t>
   </si>
@@ -89,6 +89,9 @@
   </si>
   <si>
     <t>Mallcom garment</t>
+  </si>
+  <si>
+    <t>Task 7048 : MTO Mallcom deployment GRT and Shoes with ddq fixes</t>
   </si>
 </sst>
 </file>
@@ -944,7 +947,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.54296875" bestFit="1" customWidth="1"/>
@@ -1122,6 +1125,33 @@
         <v>14</v>
       </c>
     </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
+        <v>45663</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
brandix deployment and errorhandling fixes in user creation
</commit_message>
<xml_diff>
--- a/deployment matrix/Deployment Matrix For Frontend.xlsx
+++ b/deployment matrix/Deployment Matrix For Frontend.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tarun.shetty\Desktop\VFlow\vflow-frontend\deployment matrix\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VFLOW\vflow-frontend\deployment matrix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90238C43-DF73-469D-B700-8E4767245194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A43D0224-486A-4B11-B7C3-35CEE65CC71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Matrix For Frontend" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="32">
   <si>
     <t>Date</t>
   </si>
@@ -101,6 +101,21 @@
   </si>
   <si>
     <t>Task 7133: MTO MDM filter update</t>
+  </si>
+  <si>
+    <t>Tag</t>
+  </si>
+  <si>
+    <t>develop-vflow/v1.0.0</t>
+  </si>
+  <si>
+    <t>Nilesh</t>
+  </si>
+  <si>
+    <t>Task 7600: MTO Pivot decimal fixes</t>
+  </si>
+  <si>
+    <t>Dorfketal</t>
   </si>
 </sst>
 </file>
@@ -603,12 +618,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -668,9 +684,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -708,7 +724,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -814,7 +830,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -956,7 +972,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -964,57 +980,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="57.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.81640625" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="57.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
-      </c>
-      <c r="K1">
-        <v>1</v>
       </c>
       <c r="L1" t="s">
         <v>21</v>
@@ -1025,22 +1040,22 @@
       <c r="N1" t="s">
         <v>24</v>
       </c>
+      <c r="O1" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>45643</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
       </c>
       <c r="F2" t="s">
         <v>13</v>
@@ -1048,97 +1063,100 @@
       <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="3"/>
-      <c r="J2">
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" s="3"/>
+      <c r="K2">
         <v>2</v>
       </c>
       <c r="L2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>45645</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>13</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>15</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="3"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="3"/>
       <c r="L3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>45646</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>13</v>
-      </c>
-      <c r="F4" t="s">
-        <v>15</v>
       </c>
       <c r="G4" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" t="s">
+        <v>15</v>
+      </c>
       <c r="I4" s="2"/>
-      <c r="J4">
+      <c r="J4" s="2"/>
+      <c r="K4">
         <v>2</v>
       </c>
       <c r="L4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>45660</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>13</v>
-      </c>
-      <c r="F5" t="s">
-        <v>15</v>
       </c>
       <c r="G5" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="2"/>
       <c r="L5" t="s">
         <v>14</v>
       </c>
@@ -1146,76 +1164,111 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>45663</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>11</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>23</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>13</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
       </c>
       <c r="G6" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="3"/>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
       <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>45665</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>10</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>18</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>25</v>
       </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="3"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="3"/>
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
       <c r="N7" s="4"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>45666</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>18</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>26</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>13</v>
-      </c>
-      <c r="F8" t="s">
-        <v>15</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="2"/>
+      <c r="H8" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="2"/>
       <c r="M8" s="2"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9">
+        <v>2</v>
+      </c>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
edited the deployment matrix of brandix that deployed on 31-jan
</commit_message>
<xml_diff>
--- a/deployment matrix/Deployment Matrix For Frontend.xlsx
+++ b/deployment matrix/Deployment Matrix For Frontend.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VFLOW\vflow-frontend\deployment matrix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A43D0224-486A-4B11-B7C3-35CEE65CC71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D25B12-B3CA-49A0-9784-CC940EEEA704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="34">
   <si>
     <t>Date</t>
   </si>
@@ -116,6 +116,12 @@
   </si>
   <si>
     <t>Dorfketal</t>
+  </si>
+  <si>
+    <t>develop-vflow/v1.0.1</t>
+  </si>
+  <si>
+    <t>Task 7792: MTO - Brandix download report api fix and bm report filter fix</t>
   </si>
 </sst>
 </file>
@@ -980,21 +986,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="20.81640625" customWidth="1"/>
     <col min="3" max="3" width="13.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="57.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="62.26953125" customWidth="1"/>
     <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.08984375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.81640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="11" max="11" width="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="15" max="15" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
@@ -1029,19 +1035,19 @@
         <v>8</v>
       </c>
       <c r="K1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O1" t="s">
         <v>9</v>
-      </c>
-      <c r="L1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" t="s">
-        <v>22</v>
-      </c>
-      <c r="N1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
@@ -1068,11 +1074,11 @@
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="3"/>
-      <c r="K2">
+      <c r="K2" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2">
         <v>2</v>
-      </c>
-      <c r="L2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.35">
@@ -1099,7 +1105,7 @@
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="3"/>
-      <c r="L3" t="s">
+      <c r="K3" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1127,11 +1133,11 @@
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4">
+      <c r="K4" t="s">
+        <v>19</v>
+      </c>
+      <c r="O4">
         <v>2</v>
-      </c>
-      <c r="L4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
@@ -1157,10 +1163,10 @@
         <v>15</v>
       </c>
       <c r="I5" s="2"/>
+      <c r="K5" t="s">
+        <v>14</v>
+      </c>
       <c r="L5" t="s">
-        <v>14</v>
-      </c>
-      <c r="M5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1188,8 +1194,8 @@
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
       <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
@@ -1206,9 +1212,9 @@
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="3"/>
+      <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
@@ -1233,7 +1239,7 @@
         <v>15</v>
       </c>
       <c r="I8" s="2"/>
-      <c r="M8" s="2"/>
+      <c r="L8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
@@ -1262,13 +1268,48 @@
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
-      <c r="K9">
-        <v>2</v>
-      </c>
+      <c r="K9" s="5"/>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
+        <v>45688</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="3"/>
+      <c r="O10">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>